<commit_message>
(doc): Update tableau de synthèse with new data
</commit_message>
<xml_diff>
--- a/public/excel/tableau-de-synthese.xlsx
+++ b/public/excel/tableau-de-synthese.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="41">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -383,6 +383,306 @@
 Captures SQL Developer
 Procédure Broker Portal
 Documentation du processus</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Portfolio professionnel (site web personnel)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Développement du site en React, TypeScript, Vite et Tailwind CSS
+Présentation du parcours, des compétences et des réalisations E5 / E6
+Page de veille technologique alimentée par flux RSS
+Versionnement Git / GitHub (branches, pull requests)
+Déploiement continu sur Vercel
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Site en ligne : https://thomas-montout.vercel.app/
+Dépôt GitHub
+Tableau de synthèse E5</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In the Cave – RPG textuel en React / TypeScript
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Reprise d'un exercice JavaScript freeCodeCamp comme base du projet
+Cahier des charges, maquette et modèle logique de données
+Migration progressive de JavaScript vers TypeScript
+Interface React et gestion d'état avec Zustand
+Déploiement sur Vercel
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Cahier des charges (maquette, modèle logique de données)
+Dépôt GitHub
+Application en ligne</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Absolute Stream – plateforme de suivi de films et séries (binôme)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Cahier des charges et modélisation de la base de données
+Organisation en sprints avec Trello
+Travail en binôme sous Git (branches, code review)
+Proxy API TMDB, recherche globale et pages catalogue
+Authentification sécurisée et protection des routes
+Pipeline CI GitHub Actions et tests fonctionnels manuels
+Déploiement sur Vercel
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Cahier des charges
+Documentation API et dictionnaire de données
+Scénarios de tests
+Dépôt GitHub
+Application en ligne</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">V.ROOM – e-commerce de véhicules avec assistant IA
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Cahier des charges : besoins, acteurs et répartition des droits
+Modélisation orientée objet (diagramme de classes, héritage)
+API REST Symfony 7 et persistance avec Doctrine
+Interface React avec gestion d'état Zustand
+Assistant IA côté serveur (recherche en langage naturel)
+Sécurisation des routes API, des mots de passe et de la clé d'API
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Cahier des charges
+Maquettes
+Diagramme de classes UML
+Dépôt GitHub</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pink Monster – jeu de plateforme 2D avec Phaser
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Prise en main du framework Phaser
+Programmation orientée objet appliquée au jeu vidéo
+Gestion des états du jeu
+Intégration de graphismes en pixel art
+Déploiement sur GitHub Pages
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Dépôt GitHub
+Jeu en ligne</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Site faire-part de mariage
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Conception d'un site faire-part pour un mariage
+Animations et mise en scène en React / CSS
+Mise en ligne sous un nom de domaine dédié
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Site en ligne : https://nathalieluc.fr/</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tempo – application météo
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Consommation d'une API météo publique
+Interface dont l'apparence change selon la météo
+Développement en React / TypeScript avec Vite
+Déploiement sur Vercel
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Dépôt GitHub
+Application en ligne</t>
     </r>
   </si>
 </sst>
@@ -1446,44 +1746,70 @@
       <c r="L8" s="22"/>
       <c r="M8" s="22"/>
     </row>
-    <row r="9" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="9"/>
+    <row r="9" spans="1:13" s="2" customFormat="1" ht="179.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="B9" s="8"/>
       <c r="C9" s="14"/>
       <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
+      <c r="E9" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="16"/>
+      <c r="G9" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>25</v>
+      </c>
       <c r="I9" s="22"/>
       <c r="J9" s="22"/>
       <c r="K9" s="22"/>
       <c r="L9" s="22"/>
       <c r="M9" s="22"/>
     </row>
-    <row r="10" spans="1:13" s="2" customFormat="1" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23"/>
+    <row r="10" spans="1:13" s="2" customFormat="1" ht="179.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="23" t="s">
+        <v>35</v>
+      </c>
       <c r="B10" s="8"/>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="16"/>
+      <c r="F10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>25</v>
+      </c>
       <c r="I10"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
     </row>
-    <row r="11" spans="1:13" s="2" customFormat="1" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="23"/>
+    <row r="11" spans="1:13" s="2" customFormat="1" ht="242.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="23" t="s">
+        <v>36</v>
+      </c>
       <c r="B11" s="8"/>
-      <c r="C11" s="15"/>
+      <c r="C11" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="E11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H11" s="16"/>
       <c r="I11" s="22"/>
       <c r="J11" s="22"/>
@@ -1491,13 +1817,21 @@
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
     </row>
-    <row r="12" spans="1:13" s="2" customFormat="1" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="23"/>
+    <row r="12" spans="1:13" s="2" customFormat="1" ht="210.8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="B12" s="8"/>
-      <c r="C12" s="15"/>
+      <c r="C12" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+      <c r="E12" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="G12" s="15"/>
       <c r="H12" s="16"/>
       <c r="I12"/>
@@ -1506,29 +1840,41 @@
       <c r="L12" s="22"/>
       <c r="M12" s="22"/>
     </row>
-    <row r="13" spans="1:13" s="2" customFormat="1" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="23"/>
+    <row r="13" spans="1:13" s="2" customFormat="1" ht="164.0" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="B13" s="8"/>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="16"/>
+      <c r="G13" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>25</v>
+      </c>
       <c r="I13" s="22"/>
       <c r="J13" s="22"/>
       <c r="K13" s="22"/>
       <c r="L13" s="22"/>
       <c r="M13" s="22"/>
     </row>
-    <row r="14" spans="1:13" s="2" customFormat="1" ht="69.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="23"/>
+    <row r="14" spans="1:13" s="2" customFormat="1" ht="117.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="23" t="s">
+        <v>39</v>
+      </c>
       <c r="B14" s="8"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
+      <c r="E14" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
+      <c r="G14" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H14" s="16"/>
       <c r="I14" s="22"/>
       <c r="J14" s="22"/>
@@ -1536,15 +1882,21 @@
       <c r="L14" s="22"/>
       <c r="M14" s="22"/>
     </row>
-    <row r="15" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
+    <row r="15" spans="1:13" s="2" customFormat="1" ht="148.4" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="B15" s="8"/>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="16"/>
+      <c r="G15" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>25</v>
+      </c>
       <c r="I15" s="22"/>
       <c r="J15" s="22"/>
       <c r="K15" s="22"/>

</xml_diff>

<commit_message>
Add minia-iso-stock image to the project
- Introduced a new PNG image file located at public/img/photos/minia-iso-stock.png.
</commit_message>
<xml_diff>
--- a/public/excel/tableau-de-synthese.xlsx
+++ b/public/excel/tableau-de-synthese.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="43">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -532,10 +532,11 @@
       </rPr>
       <t xml:space="preserve">Cahier des charges : besoins, acteurs et répartition des droits
 Modélisation orientée objet (diagramme de classes, héritage)
-API REST Symfony 7 et persistance avec Doctrine
+API REST Symfony 7, Doctrine et base PostgreSQL
 Interface React avec gestion d'état Zustand
 Assistant IA côté serveur (recherche en langage naturel)
 Sécurisation des routes API, des mots de passe et de la clé d'API
+Déploiement : front sur Vercel, API Docker et PostgreSQL sur Railway
 </t>
     </r>
     <r>
@@ -560,7 +561,8 @@
       <t xml:space="preserve">Cahier des charges
 Maquettes
 Diagramme de classes UML
-Dépôt GitHub</t>
+Dépôt GitHub
+Application en ligne</t>
     </r>
   </si>
   <si>
@@ -683,6 +685,97 @@
       </rPr>
       <t xml:space="preserve">Dépôt GitHub
 Application en ligne</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ISO Stock – suivi du matériel d'une flotte de véhicules
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Recueil des règles de gestion auprès d'un commanditaire réel
+Modélisation des données (MCD) et base SQLite
+Architecture en couches : interface Swing, services, DAO (JDBC)
+Stock calculé par mouvements et historique des affectations
+Import du parc depuis des fichiers CSV (28 véhicules, 81 articles)
+Tests unitaires JUnit des règles de gestion
+Livraison au client d'un exécutable autonome (jpackage)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Dépôt GitHub (README, schéma SQL commenté)
+Modèle conceptuel de données
+Tests JUnit
+Captures de l'application</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">E-enseignement – site pédagogique et vitrine (équipe de 4)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Équipe de 4 : Trello, Gantt, branches et pull requests GitHub
+Ma part : page Exercices et sa logique JavaScript (exercices.js)
+Rédaction des cours et des 6 exercices corrigés (algo, C, Java, JS, PHP)
+Uniformisation du style des pages (typographie, cartes, animations)
+README final du projet
+Mise en ligne sur GitHub Pages
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Documents et productions associés
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Cahier des charges
+Maquette, charte graphique et Gantt
+Dépôt GitHub
+Site en ligne</t>
     </r>
   </si>
 </sst>
@@ -1817,7 +1910,7 @@
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
     </row>
-    <row r="12" spans="1:13" s="2" customFormat="1" ht="210.8" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" s="2" customFormat="1" ht="242.0" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="23" t="s">
         <v>37</v>
       </c>
@@ -1832,7 +1925,9 @@
       <c r="F12" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="15"/>
+      <c r="G12" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H12" s="16"/>
       <c r="I12"/>
       <c r="J12" s="22"/>
@@ -1903,14 +1998,22 @@
       <c r="L15" s="22"/>
       <c r="M15" s="22"/>
     </row>
-    <row r="16" spans="1:13" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
+    <row r="16" spans="1:13" s="2" customFormat="1" ht="226.4" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="B16" s="8"/>
       <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
+      <c r="D16" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
+      <c r="F16" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H16" s="16"/>
       <c r="I16" s="22"/>
       <c r="J16" s="22"/>
@@ -1918,14 +2021,22 @@
       <c r="L16" s="22"/>
       <c r="M16" s="22"/>
     </row>
-    <row r="17" spans="1:8" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
+    <row r="17" spans="1:8" s="2" customFormat="1" ht="210.8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="B17" s="8"/>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
+      <c r="E17" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="H17" s="16"/>
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>